<commit_message>
Report Suite: regenerate import post-review (delta = WIP-TAB-02 + WIP-SORT-03 only, full gate re-passed) + definitive state (REVIEWED CLEAN, READY FOR USER IMPORT)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/report-suite-v1-testrail-import.xlsx
+++ b/testrail-import/report-suite-v1-testrail-import.xlsx
@@ -17587,12 +17587,13 @@
       <c r="G358" s="2" t="inlineStr">
         <is>
           <t>1. Four tabs are shown, labeled in this order: "Approved - partially completed", "Approved - not started", "Completed", and "Estimates".
-2. The "Approved - partially completed" tab is selected by default on load.</t>
+2. The "Approved - partially completed" tab is selected by default on load.
+3. There is NO on-screen status filter — the four tabs take the place of a status filter (the tab a job lands in is derived from its status and whether any work has started).</t>
         </is>
       </c>
       <c r="H358" s="2" t="inlineStr">
         <is>
-          <t>specs/wip-work-in-progress.md Story 1 S1-R2; S1-R3</t>
+          <t>specs/wip-work-in-progress.md Story 1 S1-R2; S1-R3; §3 Key Decisions (no on-screen status filter)</t>
         </is>
       </c>
       <c r="I358" s="2" t="inlineStr"/>
@@ -19191,7 +19192,7 @@
       </c>
       <c r="G391" s="2" t="inlineStr">
         <is>
-          <t>1. Money and numeric columns sort by their underlying numeric value (so $1,100.00 sorts above $900.00 ascending-wise, not alphabetically).
+          <t>1. Money and numeric columns sort by their underlying numeric value (so $1,100.00 is treated as more than $900.00, not compared as text).
 2. Days Open sorts by its day count.
 3. Status sorts by its displayed label.
 4. The Asset column sorts by unit number.

</xml_diff>